<commit_message>
Add TAM sheet to MV Electrosystems model; correct prospectus page references; log session 2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J9bdABqjFfyPGNtkJN8pfp
</commit_message>
<xml_diff>
--- a/research/MV_Electrosystems/MVELECTRO_Model_v1.xlsx
+++ b/research/MV_Electrosystems/MVELECTRO_Model_v1.xlsx
@@ -9,10 +9,11 @@
   </bookViews>
   <sheets>
     <sheet name="P&amp;L" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Quarterly" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Segments" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Valuations" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Sources" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="TAM" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Quarterly" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Segments" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Valuations" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Sources" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -406,7 +407,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="369">
   <si>
     <t xml:space="preserve">MV Electrosystems Ltd (NSE: MVELECTRO, BSE: 544851) - Model v1 (historicals). Standalone = consolidated: no subsidiary, associate or JV (FY26 AR, CARO cl. ix(e)). Rs. crore unless stated.</t>
   </si>
@@ -924,6 +925,249 @@
     <t xml:space="preserve">Memo: FY20-FY22 are Indian GAAP figures from the audited statements signed by Jugal Arora &amp; Co (FY20 figures are the comparatives in the FY21 statement). FY23 onwards Ind AS. The two bases differ (leases, ECL), so FY22 to FY23 is not strictly comparable.</t>
   </si>
   <si>
+    <t xml:space="preserve">Total addressable market (TAM), Rs. crore per year - rough first cut, 25-Oct-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built from the customer's own numbers (Indian Railways production and orders) where they exist; management unit prices from the 27-Aug-2026 call; [E] marks analyst placeholders to be replaced. Blue = input, black = formula, yellow = the base assumption that matters most.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MV status today</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Units/yr Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rs cr per unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAM Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAM Base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAM High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis and source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A. Addressable now - MV is an approved supplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Locomotive propulsion, new build (CLW, BLW, PLW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved Sep-2025; 564 sets in hand; won 27% of FY26 tenders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sets tendered per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A / S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base = sets tendered by the three railway loco works for FY26 (Prospectus p.126: programme 1,700, tendered 1,659). FY26 output ~1,700 (BLW 572 PTI 31-Mar-26; CLW incl. Dankuni 800 Rail Analysis; PLW programme 325). High = output keeps rising; Low = FY27 programme cut (one BLW FY27 target report says 468 vs 572 built). Price = PO basic rate ex GST (Pro p.26).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Locomotive propulsion, maintenance contracts (AMC) - steady state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bundled in every PO; starts after warranty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Locos under AMC per year x 3-yr fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A / E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each PO carries a 3-year AMC worth Rs.12.3 lakh per set (Pro p.26: Rs.551.22 mn / 450 sets). Steady state, three cohorts are under AMC at once, so annual AMC pool = one year's sets x full 3-yr fee. Warranty length not disclosed, so timing of first AMC revenue unknown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coach electricals: conduits, harnesses, switchgear panels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MV's legacy line; Rs.44.7 cr FY26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n.s.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not sized: no disclosure of content per coach or the competitor set. MV FY26 revenue Rs.44.7 cr (AR26 note 39) is the only hard number; utilisation fell to 46-71% on conduit lines in FY26 (Pro p.245).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. Addressable now by tender, no order yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automatic fault locators for 25 kV overhead lines (with PNC Technologies, Korea)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-yr exclusive tie-up Aug-2025; bids submitted, no win disclosed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traction-substation spans per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E / M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stock of ~1,550 substation spans (helper block below) rolled out over 5-7 years per management, priced at Rs.36/24/12 lakh per substation / sectioning / sub-sectioning locator (call 27-Aug-26). Likely partly a replacement market: fault locators already exist on many sections. High uncertainty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. Needs a new approval (12-24 months)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMU / MEMU propulsion (12-car rakes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One developmental order: 6 MEMU rakes, MCF Raebareli, Rs.86.5 cr; RDSO approval ~15-16 months away</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rakes per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A / S / M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price from the MCF LoA (Pro p.25): Rs.86.5 cr for 6 rakes = Rs.14.4 cr per rake (mgmt: ~Rs.16 cr incl. electrics). Units: 238 AC EMU rakes for Mumbai 2027-2030 (~60/yr, Statesman) plus other EMU/MEMU; mgmt says 300-500 EMUs tendered this year - unclear if rakes or cars, so used only as the high case.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D. Long-dated: incumbent OEMs, bundled supply or no programme yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vande Bharat trainset propulsion and electrics (16-car)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No order, no approval; same distributed-traction platform as EMU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S / M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price: mgmt Rs.~40 cr per 16-car rake incl. associated electrics (call). Units: ~100 Vande Bharat-platform trains built by end-2025 since 2019 (~15/yr actual); plan of 3,200 coaches for 2025-27 (~100 rakes/yr, Swarajya); 1,300 rakes sanctioned in the Rolling Stock Programme 2026-27 (Pro p.193). Base 60 = between history and plan. Much of new-generation Vande Bharat is awarded to OEM consortia that bring their own propulsion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro propulsion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No product; metro OEMs (Alstom, BEML, Titagarh, Hitachi) bundle propulsion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not sized: no national metro-car demand figure found. CareEdge (Pro p.200) puts metro + Vande Bharat + Amrit Bharat propulsion at ~USD 114 mn in CY25, i.e. ~Rs.970 cr - lower than the Vande Bharat row above because actual Vande Bharat output so far is far below plan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Locomotive propulsion retrofit (GTO-era three-phase fleet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mentioned by mgmt; no tender or RDSO programme found</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sets per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLACEHOLDER. Early WAG-9/WAP-5/WAP-7 units carry GTO converters (Wikipedia; first IGBT WAG-9 was no. 31248). No retrofit tender or count of GTO units found. 100 sets/yr at Rs.1.2 cr (converters only) is a guess to be replaced; excluded from every case total.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rest of the integrated propulsion kit (traction motors, transformer, bogies) for loco tenders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MV makes none of these; Korean motor partner (Hansung) mentioned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied from CareEdge loco market</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S / E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Railway Board directive Mar-2025: loco works to buy an integrated propulsion kit (Pro p.54, risk factor 27; p.226). CareEdge loco propulsion market USD 794.5 mn CY25 (~Rs.6,750 cr) vs ~Rs.2,720 cr for MV-type electronics bottom-up; the gap (~Rs.4,000 cr) is roughly the rest of the kit plus non-railway-works locos (Siemens 9,000 HP, Alstom 12,000 HP). Addressable only with partners.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTALS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Addressable today: approved product + open tenders (rows 6, 7, 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excludes coach electricals and metro (not sized), the retrofit placeholder, and the rest of the kit (row 17, partners only).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Plus EMU/MEMU and Vande Bharat once approved (rows 12, 14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helper: fault-locator value per substation span, Rs cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helper: substation spans rolled out per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Electrified route km / substation spacing (km) = substation spans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Roll-out period, years (mgmt: 5-7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helper: CareEdge loco propulsion market, Rs cr, less MV-type electronics base TAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Sectioning posts per substation (Prayagraj division: 33 / 29)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Sub-sectioning posts per substation (Prayagraj division: 46 / 29)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Electrified broad-gauge route km (Pro p.196)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Average substation spacing, km (Western Railway TRD: 35-50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  CareEdge India loco propulsion market CY25, USD mn (Pro p.200)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  USD/INR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What locomotive propulsion alone is worth to MV at different shares (base TAM, row 6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of sets tendered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue Rs cr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x FY26 revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;- FY26 actual share (450 / 1,659)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read-across: management's 40 sets a month = 480 sets = 29% of base tenders; today MV earns Rs.49 cr against a Rs.~2,900 cr pool it is approved for.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quarterly P&amp;L, standalone (Rs. crore). Only three quarters are public: the company listed on 6-Aug-2026. Source: Q1FY27 results filing 25-Aug-2026 (ACE quarterly dump has Q1FY26 and Q1FY27 only). Periods verified from the results table header ("Quarter ended 30-06-2026").</t>
   </si>
   <si>
@@ -1014,7 +1258,7 @@
     <t xml:space="preserve">Legacy lines YoY</t>
   </si>
   <si>
-    <t xml:space="preserve">Order book, 3-phase propulsion (as on 30-Jun-2026) [A: prospectus p.22, 125-126; PPT p.16]</t>
+    <t xml:space="preserve">Order book, 3-phase propulsion (as on 30-Jun-2026) [A: prospectus p.23, 25-26, 126; PPT p.16]</t>
   </si>
   <si>
     <t xml:space="preserve">Customer / order</t>
@@ -1083,15 +1327,12 @@
     <t xml:space="preserve">FY26 tender share: 450 of 1,659 sets tendered by CLW/BLW/PLW = 27.1% [A: prospectus p.126]</t>
   </si>
   <si>
-    <t xml:space="preserve">Capacity (single shift, chartered engineer certificate 7-Jul-2026) [A: prospectus p.240-241; PPT p.15]</t>
+    <t xml:space="preserve">Capacity (single shift, chartered engineer certificate 7-Jul-2026) [A: prospectus p.245; PPT p.15]</t>
   </si>
   <si>
     <t xml:space="preserve">Product</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit</t>
-  </si>
-  <si>
     <t xml:space="preserve">Installed capacity</t>
   </si>
   <si>
@@ -1242,7 +1483,7 @@
     <t xml:space="preserve">Prospectus</t>
   </si>
   <si>
-    <t xml:space="preserve">Prospectus dated 3-Aug-2026 (SEBI / company website): capital history p.103-106, 153; customers p.22, 218; order book p.22-26, 125-126, 216; capacity p.240-241; contingent liabilities p.85; related parties p.86; KPIs and peers p.148-153; competition p.246.</t>
+    <t xml:space="preserve">Prospectus dated 3-Aug-2026 (SEBI / company website): capital history p.104-106, 153; customers p.22, 218; order book p.23-26, 126, 216; capacity p.245; purchase orders p.26; working-capital plan p.133; LD terms p.31; contingent liabilities p.85; related parties p.86; KPIs and peers p.148-153; competition p.246.</t>
   </si>
   <si>
     <t xml:space="preserve">Q1FY27 results</t>
@@ -1279,7 +1520,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0;\(#,##0.0\);\-"/>
     <numFmt numFmtId="166" formatCode="0%"/>
@@ -1289,10 +1530,12 @@
     <numFmt numFmtId="170" formatCode="#,##0.00;\(#,##0.00\);\-"/>
     <numFmt numFmtId="171" formatCode="#,##0"/>
     <numFmt numFmtId="172" formatCode="0.0\x"/>
-    <numFmt numFmtId="173" formatCode="0.0000"/>
-    <numFmt numFmtId="174" formatCode="0.0"/>
+    <numFmt numFmtId="173" formatCode="#,##0;\(#,##0\);\-"/>
+    <numFmt numFmtId="174" formatCode="0.00"/>
+    <numFmt numFmtId="175" formatCode="0.0000"/>
+    <numFmt numFmtId="176" formatCode="0.0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1371,6 +1614,13 @@
       <family val="2"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -1385,7 +1635,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1395,13 +1645,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFC0C0C0"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -1439,7 +1695,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="64">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1548,11 +1804,67 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1580,11 +1892,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1592,7 +1904,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1600,19 +1912,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="176" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1620,11 +1932,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1632,16 +1944,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1656,7 +1964,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -5203,282 +5511,745 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="27" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
         <v>173</v>
       </c>
-      <c r="B2" s="5" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="B4" s="28" t="s">
         <v>175</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="C4" s="28" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
+      <c r="D4" s="29" t="s">
         <v>177</v>
       </c>
-      <c r="B3" s="18" t="n">
-        <v>13.448</v>
-      </c>
-      <c r="C3" s="18" t="n">
-        <v>14.933</v>
-      </c>
-      <c r="D3" s="18" t="n">
-        <v>12.771</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
+      <c r="E4" s="29" t="s">
         <v>178</v>
       </c>
-      <c r="B4" s="18" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="C4" s="18" t="n">
-        <v>0.121</v>
-      </c>
-      <c r="D4" s="18" t="n">
-        <v>0.026</v>
+      <c r="F4" s="29" t="s">
+        <v>179</v>
+      </c>
+      <c r="G4" s="29" t="s">
+        <v>180</v>
+      </c>
+      <c r="H4" s="29" t="s">
+        <v>181</v>
+      </c>
+      <c r="I4" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="J4" s="29" t="s">
+        <v>183</v>
+      </c>
+      <c r="K4" s="29" t="s">
+        <v>184</v>
+      </c>
+      <c r="L4" s="28" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="B5" s="18" t="n">
-        <v>8.977</v>
-      </c>
-      <c r="C5" s="18" t="n">
-        <v>14.275</v>
-      </c>
-      <c r="D5" s="18" t="n">
-        <v>12.326</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="B6" s="18" t="n">
-        <v>3.458</v>
-      </c>
-      <c r="C6" s="18" t="n">
-        <v>-0.451</v>
-      </c>
-      <c r="D6" s="18" t="n">
-        <v>-0.682</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>181</v>
-      </c>
-      <c r="B7" s="18" t="n">
-        <v>2.501</v>
-      </c>
-      <c r="C7" s="18" t="n">
-        <v>3.794</v>
-      </c>
-      <c r="D7" s="18" t="n">
-        <v>4.347</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="B8" s="18" t="n">
-        <v>2.002</v>
-      </c>
-      <c r="C8" s="18" t="n">
-        <v>3.166</v>
-      </c>
-      <c r="D8" s="18" t="n">
-        <v>2.155</v>
+      <c r="A5" s="30" t="s">
+        <v>186</v>
+      </c>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+    </row>
+    <row r="6" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>188</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>189</v>
+      </c>
+      <c r="D6" s="33" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E6" s="34" t="n">
+        <v>1659</v>
+      </c>
+      <c r="F6" s="33" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G6" s="35" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="H6" s="36" t="n">
+        <f aca="false">IF(OR(D6="",G6=""),"n.s.",D6*G6)</f>
+        <v>2460</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <f aca="false">IF(OR(E6="",G6=""),"n.s.",E6*G6)</f>
+        <v>2720.76</v>
+      </c>
+      <c r="J6" s="36" t="n">
+        <f aca="false">IF(OR(F6="",G6=""),"n.s.",F6*G6)</f>
+        <v>3116</v>
+      </c>
+      <c r="K6" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E7" s="34" t="n">
+        <v>1659</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G7" s="38" t="n">
+        <f aca="false">0.1225</f>
+        <v>0.1225</v>
+      </c>
+      <c r="H7" s="36" t="n">
+        <f aca="false">IF(OR(D7="",G7=""),"n.s.",D7*G7)</f>
+        <v>183.75</v>
+      </c>
+      <c r="I7" s="37" t="n">
+        <f aca="false">IF(OR(E7="",G7=""),"n.s.",E7*G7)</f>
+        <v>203.2275</v>
+      </c>
+      <c r="J7" s="36" t="n">
+        <f aca="false">IF(OR(F7="",G7=""),"n.s.",F7*G7)</f>
+        <v>232.75</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="32" t="s">
+        <v>197</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>198</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="D8" s="33"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="36" t="str">
+        <f aca="false">IF(OR(D8="",G8=""),"n.s.",D8*G8)</f>
+        <v>n.s.</v>
+      </c>
+      <c r="I8" s="37" t="str">
+        <f aca="false">IF(OR(E8="",G8=""),"n.s.",E8*G8)</f>
+        <v>n.s.</v>
+      </c>
+      <c r="J8" s="36" t="str">
+        <f aca="false">IF(OR(F8="",G8=""),"n.s.",F8*G8)</f>
+        <v>n.s.</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="30" t="s">
+        <v>202</v>
+      </c>
+      <c r="B9" s="31"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
+    </row>
+    <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="32" t="s">
+        <v>203</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>205</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <f aca="false">E22*0.7</f>
+        <v>181.183333333333</v>
+      </c>
+      <c r="E10" s="39" t="n">
+        <f aca="false">E22</f>
+        <v>258.833333333333</v>
+      </c>
+      <c r="F10" s="36" t="n">
+        <f aca="false">E22*1.4</f>
+        <v>362.366666666667</v>
+      </c>
+      <c r="G10" s="38" t="n">
+        <f aca="false">E21</f>
+        <v>0.823448275862069</v>
+      </c>
+      <c r="H10" s="36" t="n">
+        <f aca="false">IF(OR(D10="",G10=""),"n.s.",D10*G10)</f>
+        <v>149.195103448276</v>
+      </c>
+      <c r="I10" s="37" t="n">
+        <f aca="false">IF(OR(E10="",G10=""),"n.s.",E10*G10)</f>
+        <v>213.135862068965</v>
+      </c>
+      <c r="J10" s="36" t="n">
+        <f aca="false">IF(OR(F10="",G10=""),"n.s.",F10*G10)</f>
+        <v>298.390206896552</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="30" t="s">
+        <v>208</v>
+      </c>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
+    </row>
+    <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="32" t="s">
+        <v>209</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>210</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>211</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <v>80</v>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>120</v>
+      </c>
+      <c r="F12" s="33" t="n">
+        <v>250</v>
+      </c>
+      <c r="G12" s="38" t="n">
+        <f aca="false">86.546/6</f>
+        <v>14.4243333333333</v>
+      </c>
+      <c r="H12" s="36" t="n">
+        <f aca="false">IF(OR(D12="",G12=""),"n.s.",D12*G12)</f>
+        <v>1153.94666666667</v>
+      </c>
+      <c r="I12" s="37" t="n">
+        <f aca="false">IF(OR(E12="",G12=""),"n.s.",E12*G12)</f>
+        <v>1730.92</v>
+      </c>
+      <c r="J12" s="36" t="n">
+        <f aca="false">IF(OR(F12="",G12=""),"n.s.",F12*G12)</f>
+        <v>3606.08333333333</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="30" t="s">
+        <v>214</v>
+      </c>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
+    </row>
+    <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32" t="s">
+        <v>215</v>
+      </c>
+      <c r="B14" s="32" t="s">
+        <v>216</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>211</v>
+      </c>
+      <c r="D14" s="33" t="n">
         <v>30</v>
       </c>
-      <c r="B9" s="19" t="n">
-        <f aca="false">B3-B5-B6-B7-B8</f>
-        <v>-3.49</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <f aca="false">C3-C5-C6-C7-C8</f>
-        <v>-5.851</v>
-      </c>
-      <c r="D9" s="19" t="n">
-        <f aca="false">D3-D5-D6-D7-D8</f>
-        <v>-5.375</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="B10" s="14" t="n">
-        <f aca="false">B9/B3</f>
-        <v>-0.259518143961927</v>
-      </c>
-      <c r="C10" s="14" t="n">
-        <f aca="false">C9/C3</f>
-        <v>-0.39181678162459</v>
-      </c>
-      <c r="D10" s="14" t="n">
-        <f aca="false">D9/D3</f>
-        <v>-0.420875420875421</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="18" t="n">
-        <v>0.743</v>
-      </c>
-      <c r="C11" s="18" t="n">
-        <v>1.063</v>
-      </c>
-      <c r="D11" s="18" t="n">
-        <v>1.512</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="B12" s="18" t="n">
-        <v>0.762</v>
-      </c>
-      <c r="C12" s="18" t="n">
-        <v>1.133</v>
-      </c>
-      <c r="D12" s="18" t="n">
-        <v>1.178</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="19" t="n">
-        <f aca="false">B9+B4-B11-B12</f>
-        <v>-4.93</v>
-      </c>
-      <c r="C13" s="19" t="n">
-        <f aca="false">C9+C4-C11-C12</f>
-        <v>-7.926</v>
-      </c>
-      <c r="D13" s="19" t="n">
-        <f aca="false">D9+D4-D11-D12</f>
-        <v>-8.039</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="B14" s="18" t="n">
-        <v>0.804</v>
-      </c>
-      <c r="C14" s="18" t="n">
-        <v>-5.014</v>
-      </c>
-      <c r="D14" s="18" t="n">
-        <v>-1.152</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="E14" s="34" t="n">
+        <v>60</v>
+      </c>
+      <c r="F14" s="33" t="n">
+        <v>120</v>
+      </c>
+      <c r="G14" s="35" t="n">
         <v>40</v>
       </c>
-      <c r="B15" s="19" t="n">
-        <f aca="false">B13-B14</f>
-        <v>-5.734</v>
-      </c>
-      <c r="C15" s="19" t="n">
-        <f aca="false">C13-C14</f>
-        <v>-2.912</v>
-      </c>
-      <c r="D15" s="19" t="n">
-        <f aca="false">D13-D14</f>
-        <v>-6.887</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="B16" s="14" t="n">
-        <f aca="false">B15/B3</f>
-        <v>-0.426383105294468</v>
-      </c>
-      <c r="C16" s="14" t="n">
-        <f aca="false">C15/C3</f>
-        <v>-0.195004352775732</v>
-      </c>
-      <c r="D16" s="14" t="n">
-        <f aca="false">D15/D3</f>
-        <v>-0.539268655547725</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>-5.733</v>
-      </c>
-      <c r="C17" s="18" t="n">
-        <v>-2.913</v>
-      </c>
-      <c r="D17" s="18" t="n">
-        <v>-6.886</v>
+      <c r="H14" s="36" t="n">
+        <f aca="false">IF(OR(D14="",G14=""),"n.s.",D14*G14)</f>
+        <v>1200</v>
+      </c>
+      <c r="I14" s="37" t="n">
+        <f aca="false">IF(OR(E14="",G14=""),"n.s.",E14*G14)</f>
+        <v>2400</v>
+      </c>
+      <c r="J14" s="36" t="n">
+        <f aca="false">IF(OR(F14="",G14=""),"n.s.",F14*G14)</f>
+        <v>4800</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="32" t="s">
+        <v>219</v>
+      </c>
+      <c r="B15" s="32" t="s">
+        <v>220</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="D15" s="33"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="36" t="str">
+        <f aca="false">IF(OR(D15="",G15=""),"n.s.",D15*G15)</f>
+        <v>n.s.</v>
+      </c>
+      <c r="I15" s="37" t="str">
+        <f aca="false">IF(OR(E15="",G15=""),"n.s.",E15*G15)</f>
+        <v>n.s.</v>
+      </c>
+      <c r="J15" s="36" t="str">
+        <f aca="false">IF(OR(F15="",G15=""),"n.s.",F15*G15)</f>
+        <v>n.s.</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="32" t="s">
+        <v>222</v>
+      </c>
+      <c r="B16" s="32" t="s">
+        <v>223</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>224</v>
+      </c>
+      <c r="D16" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="34" t="n">
+        <v>100</v>
+      </c>
+      <c r="F16" s="33" t="n">
+        <v>200</v>
+      </c>
+      <c r="G16" s="35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H16" s="36" t="n">
+        <f aca="false">IF(OR(D16="",G16=""),"n.s.",D16*G16)</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="37" t="n">
+        <f aca="false">IF(OR(E16="",G16=""),"n.s.",E16*G16)</f>
+        <v>120</v>
+      </c>
+      <c r="J16" s="36" t="n">
+        <f aca="false">IF(OR(F16="",G16=""),"n.s.",F16*G16)</f>
+        <v>240</v>
+      </c>
+      <c r="K16" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="36.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="32" t="s">
+        <v>227</v>
+      </c>
+      <c r="B17" s="32" t="s">
+        <v>228</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>229</v>
+      </c>
+      <c r="D17" s="33"/>
+      <c r="E17" s="39" t="n">
+        <f aca="false">E25</f>
+        <v>4032.49</v>
+      </c>
+      <c r="F17" s="33"/>
+      <c r="G17" s="38" t="n">
+        <f aca="false">1</f>
+        <v>1</v>
+      </c>
+      <c r="H17" s="36" t="str">
+        <f aca="false">IF(OR(D17="",G17=""),"n.s.",D17*G17)</f>
+        <v>n.s.</v>
+      </c>
+      <c r="I17" s="37" t="n">
+        <f aca="false">IF(OR(E17="",G17=""),"n.s.",E17*G17)</f>
+        <v>4032.49</v>
+      </c>
+      <c r="J17" s="36" t="str">
+        <f aca="false">IF(OR(F17="",G17=""),"n.s.",F17*G17)</f>
+        <v>n.s.</v>
+      </c>
+      <c r="K17" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="B18" s="21" t="n">
-        <f aca="false">B15-B17</f>
-        <v>-0.00100000000000033</v>
-      </c>
-      <c r="C18" s="21" t="n">
-        <f aca="false">C15-C17</f>
-        <v>0.00099999999999989</v>
-      </c>
-      <c r="D18" s="21" t="n">
-        <f aca="false">D15-D17</f>
-        <v>-0.00100000000000122</v>
+      <c r="A18" s="30" t="s">
+        <v>232</v>
+      </c>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+      <c r="L18" s="31"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="H19" s="37" t="n">
+        <f aca="false">H6+H7+H10</f>
+        <v>2792.94510344828</v>
+      </c>
+      <c r="I19" s="37" t="n">
+        <f aca="false">I6+I7+I10</f>
+        <v>3137.12336206897</v>
+      </c>
+      <c r="J19" s="37" t="n">
+        <f aca="false">J6+J7+J10</f>
+        <v>3647.14020689655</v>
+      </c>
+      <c r="L19" s="26" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="26" t="s">
-        <v>189</v>
+      <c r="A20" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="H20" s="37" t="n">
+        <f aca="false">H19+H12+H14</f>
+        <v>5146.89177011494</v>
+      </c>
+      <c r="I20" s="37" t="n">
+        <f aca="false">I19+I12+I14</f>
+        <v>7268.04336206897</v>
+      </c>
+      <c r="J20" s="37" t="n">
+        <f aca="false">J19+J12+J14</f>
+        <v>12053.2235402299</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="26" t="s">
-        <v>190</v>
+      <c r="A21" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="E21" s="38" t="n">
+        <f aca="false">(36+E26*24+E27*12)/100</f>
+        <v>0.823448275862069</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="E22" s="36" t="n">
+        <f aca="false">E23/E24</f>
+        <v>258.833333333333</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="E23" s="36" t="n">
+        <f aca="false">ROUND(E28/E29,0)</f>
+        <v>1553</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="E24" s="33" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="E25" s="36" t="n">
+        <f aca="false">E30*E31/10-I6</f>
+        <v>4032.49</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="E26" s="38" t="n">
+        <f aca="false">33/29</f>
+        <v>1.13793103448276</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="E27" s="38" t="n">
+        <f aca="false">46/29</f>
+        <v>1.58620689655172</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="E28" s="33" t="n">
+        <v>69873</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="E29" s="33" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>794.5</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="E31" s="33" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="30" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="40" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D35" s="36" t="n">
+        <f aca="false">ROUND(A35*$E$6,0)</f>
+        <v>249</v>
+      </c>
+      <c r="E35" s="36" t="n">
+        <f aca="false">D35*$G$6</f>
+        <v>408.36</v>
+      </c>
+      <c r="F35" s="24" t="n">
+        <f aca="false">E35/'P&amp;L'!H3</f>
+        <v>8.26171400825443</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="40" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D36" s="36" t="n">
+        <f aca="false">ROUND(A36*$E$6,0)</f>
+        <v>332</v>
+      </c>
+      <c r="E36" s="36" t="n">
+        <f aca="false">D36*$G$6</f>
+        <v>544.48</v>
+      </c>
+      <c r="F36" s="24" t="n">
+        <f aca="false">E36/'P&amp;L'!H3</f>
+        <v>11.0156186776726</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D37" s="36" t="n">
+        <f aca="false">ROUND(A37*$E$6,0)</f>
+        <v>415</v>
+      </c>
+      <c r="E37" s="36" t="n">
+        <f aca="false">D37*$G$6</f>
+        <v>680.6</v>
+      </c>
+      <c r="F37" s="24" t="n">
+        <f aca="false">E37/'P&amp;L'!H3</f>
+        <v>13.7695233470907</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="40" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="D38" s="36" t="n">
+        <f aca="false">ROUND(A38*$E$6,0)</f>
+        <v>450</v>
+      </c>
+      <c r="E38" s="36" t="n">
+        <f aca="false">D38*$G$6</f>
+        <v>738</v>
+      </c>
+      <c r="F38" s="24" t="n">
+        <f aca="false">E38/'P&amp;L'!H3</f>
+        <v>14.9308084486526</v>
+      </c>
+      <c r="G38" s="26" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="40" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D39" s="36" t="n">
+        <f aca="false">ROUND(A39*$E$6,0)</f>
+        <v>498</v>
+      </c>
+      <c r="E39" s="36" t="n">
+        <f aca="false">D39*$G$6</f>
+        <v>816.72</v>
+      </c>
+      <c r="F39" s="24" t="n">
+        <f aca="false">E39/'P&amp;L'!H3</f>
+        <v>16.5234280165089</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="26" t="s">
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -5497,522 +6268,282 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>191</v>
+        <v>253</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="41" t="s">
+        <v>254</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
-        <v>173</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>13</v>
+      <c r="A3" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="B3" s="18" t="n">
+        <v>13.448</v>
+      </c>
+      <c r="C3" s="18" t="n">
+        <v>14.933</v>
+      </c>
+      <c r="D3" s="18" t="n">
+        <v>12.771</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>194</v>
+        <v>259</v>
       </c>
       <c r="B4" s="18" t="n">
-        <v>45.7</v>
+        <v>0.065</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>33.214</v>
+        <v>0.121</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <v>0.026</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>195</v>
+        <v>260</v>
       </c>
       <c r="B5" s="18" t="n">
-        <v>16.486</v>
+        <v>8.977</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>7.879</v>
+        <v>14.275</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>12.326</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>196</v>
+        <v>261</v>
       </c>
       <c r="B6" s="18" t="n">
-        <v>0.45</v>
+        <v>3.458</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>3.627</v>
+        <v>-0.451</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>-0.682</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>197</v>
+        <v>262</v>
       </c>
       <c r="B7" s="18" t="n">
-        <v>0</v>
+        <v>2.501</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>4.708</v>
+        <v>3.794</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>4.347</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="B8" s="19" t="n">
-        <f aca="false">SUM(B4:B7)</f>
-        <v>62.636</v>
-      </c>
-      <c r="C8" s="19" t="n">
-        <f aca="false">SUM(C4:C7)</f>
-        <v>49.428</v>
+      <c r="A8" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>2.002</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>3.166</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>2.155</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="B9" s="21" t="n">
-        <f aca="false">B8-'P&amp;L'!G3</f>
-        <v>-0.000999999999997669</v>
-      </c>
-      <c r="C9" s="21" t="n">
-        <f aca="false">C8-'P&amp;L'!H3</f>
-        <v>0</v>
+      <c r="A9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="19" t="n">
+        <f aca="false">B3-B5-B6-B7-B8</f>
+        <v>-3.49</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <f aca="false">C3-C5-C6-C7-C8</f>
+        <v>-5.851</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <f aca="false">D3-D5-D6-D7-D8</f>
+        <v>-5.375</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="B10" s="28" t="n">
-        <f aca="false">B7/B8</f>
-        <v>0</v>
-      </c>
-      <c r="C10" s="28" t="n">
-        <f aca="false">C7/C8</f>
-        <v>0.095249656065388</v>
+        <v>264</v>
+      </c>
+      <c r="B10" s="14" t="n">
+        <f aca="false">B9/B3</f>
+        <v>-0.259518143961927</v>
+      </c>
+      <c r="C10" s="14" t="n">
+        <f aca="false">C9/C3</f>
+        <v>-0.39181678162459</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <f aca="false">D9/D3</f>
+        <v>-0.420875420875421</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="C11" s="28" t="n">
-        <f aca="false">SUM(C4:C6)/SUM(B4:B6)-1</f>
-        <v>-0.286033590906188</v>
+        <v>33</v>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>1.063</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>1.512</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="B12" s="18" t="n">
+        <v>0.762</v>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>1.133</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>1.178</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="s">
-        <v>203</v>
-      </c>
-      <c r="B14" s="30" t="s">
-        <v>204</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>205</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>206</v>
-      </c>
-      <c r="E14" s="30" t="s">
-        <v>207</v>
-      </c>
-      <c r="F14" s="30" t="s">
-        <v>208</v>
-      </c>
-      <c r="G14" s="30" t="s">
-        <v>209</v>
+      <c r="A13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="19" t="n">
+        <f aca="false">B9+B4-B11-B12</f>
+        <v>-4.93</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <f aca="false">C9+C4-C11-C12</f>
+        <v>-7.926</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <f aca="false">D9+D4-D11-D12</f>
+        <v>-8.039</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>0.804</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>-5.014</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>-1.152</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>210</v>
-      </c>
-      <c r="B15" s="31" t="s">
-        <v>211</v>
-      </c>
-      <c r="C15" s="32" t="n">
-        <v>200</v>
-      </c>
-      <c r="D15" s="16" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="E15" s="20" t="n">
-        <f aca="false">C15*D15</f>
-        <v>328</v>
-      </c>
-      <c r="F15" s="18" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="G15" s="20" t="n">
-        <f aca="false">E15+F15</f>
-        <v>352.6</v>
+      <c r="A15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="19" t="n">
+        <f aca="false">B13-B14</f>
+        <v>-5.734</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <f aca="false">C13-C14</f>
+        <v>-2.912</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <f aca="false">D13-D14</f>
+        <v>-6.887</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="B16" s="31" t="s">
-        <v>213</v>
-      </c>
-      <c r="C16" s="32" t="n">
-        <v>161</v>
-      </c>
-      <c r="D16" s="16" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="E16" s="20" t="n">
-        <f aca="false">C16*D16</f>
-        <v>264.04</v>
-      </c>
-      <c r="F16" s="18" t="n">
-        <v>19.803</v>
-      </c>
-      <c r="G16" s="20" t="n">
-        <f aca="false">E16+F16</f>
-        <v>283.843</v>
+        <v>267</v>
+      </c>
+      <c r="B16" s="14" t="n">
+        <f aca="false">B15/B3</f>
+        <v>-0.426383105294468</v>
+      </c>
+      <c r="C16" s="14" t="n">
+        <f aca="false">C15/C3</f>
+        <v>-0.195004352775732</v>
+      </c>
+      <c r="D16" s="14" t="n">
+        <f aca="false">D15/D3</f>
+        <v>-0.539268655547725</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>214</v>
-      </c>
-      <c r="B17" s="31" t="s">
-        <v>215</v>
-      </c>
-      <c r="C17" s="32" t="n">
-        <v>76</v>
-      </c>
-      <c r="D17" s="16" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="E17" s="20" t="n">
-        <f aca="false">C17*D17</f>
-        <v>125.4</v>
-      </c>
-      <c r="F17" s="18" t="n">
-        <v>9.12</v>
-      </c>
-      <c r="G17" s="20" t="n">
-        <f aca="false">E17+F17</f>
-        <v>134.52</v>
+        <v>268</v>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>-5.733</v>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>-2.913</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>-6.886</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="B18" s="31" t="s">
-        <v>216</v>
-      </c>
-      <c r="C18" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="D18" s="16" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="E18" s="20" t="n">
-        <f aca="false">C18*D18</f>
-        <v>21.32</v>
-      </c>
-      <c r="F18" s="18" t="n">
-        <v>1.599</v>
-      </c>
-      <c r="G18" s="20" t="n">
-        <f aca="false">E18+F18</f>
-        <v>22.919</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="B19" s="31" t="s">
-        <v>218</v>
-      </c>
-      <c r="C19" s="32" t="n">
-        <v>114</v>
-      </c>
-      <c r="D19" s="33" t="n">
-        <f aca="false">E19/C19</f>
-        <v>1.60421052631579</v>
-      </c>
-      <c r="E19" s="20" t="n">
-        <f aca="false">921.64-SUM(E15:E18)</f>
-        <v>182.88</v>
-      </c>
-      <c r="F19" s="20" t="n">
-        <f aca="false">67.678-SUM(F15:F18)</f>
-        <v>12.556</v>
-      </c>
-      <c r="G19" s="20" t="n">
-        <f aca="false">E19+F19</f>
-        <v>195.436</v>
+        <v>269</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <f aca="false">B15-B17</f>
+        <v>-0.00100000000000033</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <f aca="false">C15-C17</f>
+        <v>0.00099999999999989</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <f aca="false">D15-D17</f>
+        <v>-0.00100000000000122</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="C20" s="23" t="n">
-        <f aca="false">SUM(C15:C19)</f>
-        <v>564</v>
-      </c>
-      <c r="E20" s="19" t="n">
-        <f aca="false">SUM(E15:E19)</f>
-        <v>921.64</v>
-      </c>
-      <c r="F20" s="19" t="n">
-        <f aca="false">SUM(F15:F19)</f>
-        <v>67.678</v>
-      </c>
-      <c r="G20" s="19" t="n">
-        <f aca="false">SUM(G15:G19)</f>
-        <v>989.318</v>
+      <c r="A20" s="26" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="C21" s="34" t="n">
-        <v>8</v>
-      </c>
-      <c r="E21" s="18" t="n">
-        <v>89.86</v>
-      </c>
-      <c r="F21" s="18" t="n">
-        <v>4.87</v>
-      </c>
-      <c r="G21" s="35" t="n">
-        <f aca="false">E21+F21</f>
-        <v>94.73</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="E22" s="18" t="n">
-        <v>20</v>
-      </c>
-      <c r="G22" s="35" t="n">
-        <f aca="false">E22</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="E23" s="19" t="n">
-        <f aca="false">E20+E21+E22</f>
-        <v>1031.5</v>
-      </c>
-      <c r="G23" s="19" t="n">
-        <f aca="false">G20+G21+G22</f>
-        <v>1104.048</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="E24" s="36" t="n">
-        <f aca="false">E23/'P&amp;L'!H3</f>
-        <v>20.8687383669175</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="37" t="s">
-        <v>226</v>
-      </c>
-      <c r="B28" s="37" t="s">
-        <v>227</v>
-      </c>
-      <c r="C28" s="37" t="s">
-        <v>228</v>
-      </c>
-      <c r="D28" s="37" t="s">
-        <v>229</v>
-      </c>
-      <c r="E28" s="37" t="s">
-        <v>230</v>
-      </c>
-      <c r="F28" s="37" t="s">
-        <v>231</v>
-      </c>
-      <c r="G28" s="37" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="C29" s="32" t="n">
-        <v>1650</v>
-      </c>
-      <c r="D29" s="32" t="n">
-        <v>1650</v>
-      </c>
-      <c r="E29" s="32" t="n">
-        <v>1623</v>
-      </c>
-      <c r="F29" s="32" t="n">
-        <v>1650</v>
-      </c>
-      <c r="G29" s="14" t="n">
-        <f aca="false">F29/C29</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="C30" s="32" t="n">
-        <v>1950000</v>
-      </c>
-      <c r="D30" s="32" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="E30" s="32" t="n">
-        <v>1650000</v>
-      </c>
-      <c r="F30" s="32" t="n">
-        <v>900700</v>
-      </c>
-      <c r="G30" s="14" t="n">
-        <f aca="false">F30/C30</f>
-        <v>0.461897435897436</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="C31" s="32" t="n">
-        <v>225000</v>
-      </c>
-      <c r="D31" s="32" t="n">
-        <v>185000</v>
-      </c>
-      <c r="E31" s="32" t="n">
-        <v>210000</v>
-      </c>
-      <c r="F31" s="32" t="n">
-        <v>114632</v>
-      </c>
-      <c r="G31" s="14" t="n">
-        <f aca="false">F31/C31</f>
-        <v>0.509475555555556</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="C32" s="32" t="n">
-        <v>660000</v>
-      </c>
-      <c r="D32" s="32" t="n">
-        <v>580000</v>
-      </c>
-      <c r="E32" s="32" t="n">
-        <v>570000</v>
-      </c>
-      <c r="F32" s="32" t="n">
-        <v>472000</v>
-      </c>
-      <c r="G32" s="14" t="n">
-        <f aca="false">F32/C32</f>
-        <v>0.715151515151515</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="C33" s="32" t="n">
-        <v>114</v>
-      </c>
-      <c r="D33" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="G33" s="14" t="n">
-        <f aca="false">F33/C33</f>
-        <v>0.0263157894736842</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="26" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="26" t="s">
-        <v>242</v>
+      <c r="A21" s="26" t="s">
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -6031,233 +6562,522 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:C31"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="38" t="s">
-        <v>243</v>
-      </c>
-      <c r="C2" s="39" t="n">
-        <v>788</v>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="38" t="s">
-        <v>244</v>
-      </c>
-      <c r="C3" s="40" t="n">
-        <v>2.7283</v>
+      <c r="A3" s="41" t="s">
+        <v>254</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="38" t="s">
-        <v>245</v>
-      </c>
-      <c r="C4" s="41" t="n">
-        <f aca="false">C2*C3</f>
-        <v>2149.9004</v>
+      <c r="A4" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="B4" s="18" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="C4" s="18" t="n">
+        <v>33.214</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="38" t="s">
-        <v>246</v>
-      </c>
-      <c r="C5" s="34" t="n">
-        <v>425</v>
+      <c r="A5" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>16.486</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>7.879</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="38" t="s">
-        <v>247</v>
-      </c>
-      <c r="C6" s="42" t="n">
-        <v>273.5</v>
+      <c r="A6" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>3.627</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="38" t="s">
-        <v>248</v>
-      </c>
-      <c r="C7" s="43" t="n">
-        <f aca="false">'P&amp;L'!H180</f>
-        <v>49.715</v>
+      <c r="A7" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>4.708</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="38" t="s">
-        <v>249</v>
-      </c>
-      <c r="C8" s="34" t="n">
+      <c r="A8" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="B8" s="19" t="n">
+        <f aca="false">SUM(B4:B7)</f>
+        <v>62.636</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <f aca="false">SUM(C4:C7)</f>
+        <v>49.428</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <f aca="false">B8-'P&amp;L'!G3</f>
+        <v>-0.000999999999997669</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <f aca="false">C8-'P&amp;L'!H3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="B10" s="42" t="n">
+        <f aca="false">B7/B8</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="42" t="n">
+        <f aca="false">C7/C8</f>
+        <v>0.095249656065388</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="C11" s="42" t="n">
+        <f aca="false">SUM(C4:C6)/SUM(B4:B6)-1</f>
+        <v>-0.286033590906188</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="43" t="s">
+        <v>284</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>285</v>
+      </c>
+      <c r="C14" s="44" t="s">
+        <v>286</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>287</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>288</v>
+      </c>
+      <c r="F14" s="44" t="s">
+        <v>289</v>
+      </c>
+      <c r="G14" s="44" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="38" t="s">
-        <v>250</v>
-      </c>
-      <c r="C9" s="44" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="38" t="s">
-        <v>251</v>
-      </c>
-      <c r="C10" s="35" t="n">
-        <f aca="false">C8-C9-C7</f>
-        <v>218.285</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="38" t="s">
-        <v>252</v>
-      </c>
-      <c r="C11" s="41" t="n">
-        <f aca="false">C4-C10</f>
-        <v>1931.6154</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="4" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="38" t="s">
-        <v>254</v>
-      </c>
-      <c r="C14" s="36" t="n">
-        <f aca="false">C11/'P&amp;L'!H3</f>
-        <v>39.079376062151</v>
-      </c>
-    </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="38" t="s">
-        <v>255</v>
-      </c>
-      <c r="C15" s="36" t="n">
-        <f aca="false">C2/129.23</f>
-        <v>6.09765534318657</v>
+      <c r="A15" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="B15" s="45" t="s">
+        <v>292</v>
+      </c>
+      <c r="C15" s="46" t="n">
+        <v>200</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <f aca="false">C15*D15</f>
+        <v>328</v>
+      </c>
+      <c r="F15" s="18" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G15" s="20" t="n">
+        <f aca="false">E15+F15</f>
+        <v>352.6</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="38" t="s">
-        <v>256</v>
-      </c>
-      <c r="C16" s="45" t="s">
-        <v>257</v>
+      <c r="A16" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="B16" s="45" t="s">
+        <v>294</v>
+      </c>
+      <c r="C16" s="46" t="n">
+        <v>161</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <f aca="false">C16*D16</f>
+        <v>264.04</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>19.803</v>
+      </c>
+      <c r="G16" s="20" t="n">
+        <f aca="false">E16+F16</f>
+        <v>283.843</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="B17" s="45" t="s">
+        <v>296</v>
+      </c>
+      <c r="C17" s="46" t="n">
+        <v>76</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <f aca="false">C17*D17</f>
+        <v>125.4</v>
+      </c>
+      <c r="F17" s="18" t="n">
+        <v>9.12</v>
+      </c>
+      <c r="G17" s="20" t="n">
+        <f aca="false">E17+F17</f>
+        <v>134.52</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="4" t="s">
-        <v>258</v>
+      <c r="A18" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="B18" s="45" t="s">
+        <v>297</v>
+      </c>
+      <c r="C18" s="46" t="n">
+        <v>13</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <f aca="false">C18*D18</f>
+        <v>21.32</v>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>1.599</v>
+      </c>
+      <c r="G18" s="20" t="n">
+        <f aca="false">E18+F18</f>
+        <v>22.919</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="38" t="s">
-        <v>259</v>
-      </c>
-      <c r="C19" s="44" t="n">
-        <v>40</v>
+      <c r="A19" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="B19" s="45" t="s">
+        <v>299</v>
+      </c>
+      <c r="C19" s="46" t="n">
+        <v>114</v>
+      </c>
+      <c r="D19" s="47" t="n">
+        <f aca="false">E19/C19</f>
+        <v>1.60421052631579</v>
+      </c>
+      <c r="E19" s="20" t="n">
+        <f aca="false">921.64-SUM(E15:E18)</f>
+        <v>182.88</v>
+      </c>
+      <c r="F19" s="20" t="n">
+        <f aca="false">67.678-SUM(F15:F18)</f>
+        <v>12.556</v>
+      </c>
+      <c r="G19" s="20" t="n">
+        <f aca="false">E19+F19</f>
+        <v>195.436</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="38" t="s">
-        <v>260</v>
-      </c>
-      <c r="C20" s="44" t="n">
-        <v>1.64</v>
+      <c r="A20" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="C20" s="23" t="n">
+        <f aca="false">SUM(C15:C19)</f>
+        <v>564</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <f aca="false">SUM(E15:E19)</f>
+        <v>921.64</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <f aca="false">SUM(F15:F19)</f>
+        <v>67.678</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <f aca="false">SUM(G15:G19)</f>
+        <v>989.318</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="38" t="s">
-        <v>261</v>
-      </c>
-      <c r="C21" s="41" t="n">
-        <f aca="false">C19*12*C20</f>
-        <v>787.2</v>
+      <c r="A21" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="C21" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>89.86</v>
+      </c>
+      <c r="F21" s="18" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="G21" s="49" t="n">
+        <f aca="false">E21+F21</f>
+        <v>94.73</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="38" t="s">
-        <v>262</v>
-      </c>
-      <c r="C22" s="46" t="n">
-        <f aca="false">SUM(Segments!C4:C6)</f>
-        <v>44.72</v>
+      <c r="A22" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="G22" s="49" t="n">
+        <f aca="false">E22</f>
+        <v>20</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="38" t="s">
-        <v>263</v>
-      </c>
-      <c r="C23" s="41" t="n">
-        <f aca="false">C21+C22</f>
-        <v>831.92</v>
+      <c r="A23" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <f aca="false">E20+E21+E22</f>
+        <v>1031.5</v>
+      </c>
+      <c r="G23" s="19" t="n">
+        <f aca="false">G20+G21+G22</f>
+        <v>1104.048</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="38" t="s">
-        <v>264</v>
-      </c>
-      <c r="C24" s="47" t="n">
-        <v>0.1</v>
+      <c r="A24" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="E24" s="50" t="n">
+        <f aca="false">E23/'P&amp;L'!H3</f>
+        <v>20.8687383669175</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="38" t="s">
-        <v>265</v>
-      </c>
-      <c r="C25" s="41" t="n">
-        <f aca="false">C23*C24</f>
-        <v>83.192</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="38" t="s">
-        <v>266</v>
-      </c>
-      <c r="C26" s="36" t="n">
-        <f aca="false">C4/C25</f>
-        <v>25.8426339071065</v>
+      <c r="A25" s="26" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="38" t="s">
-        <v>267</v>
-      </c>
-      <c r="C27" s="41" t="n">
-        <f aca="false">C19*12</f>
-        <v>480</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="38" t="s">
-        <v>268</v>
-      </c>
-      <c r="C28" s="48" t="n">
-        <f aca="false">Segments!C20/C27*12</f>
-        <v>14.1</v>
+      <c r="A27" s="4" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="51" t="s">
+        <v>307</v>
+      </c>
+      <c r="B28" s="51" t="s">
+        <v>176</v>
+      </c>
+      <c r="C28" s="51" t="s">
+        <v>308</v>
+      </c>
+      <c r="D28" s="51" t="s">
+        <v>309</v>
+      </c>
+      <c r="E28" s="51" t="s">
+        <v>310</v>
+      </c>
+      <c r="F28" s="51" t="s">
+        <v>311</v>
+      </c>
+      <c r="G28" s="51" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="38" t="s">
-        <v>269</v>
-      </c>
-      <c r="C29" s="49" t="n">
-        <f aca="false">450/C27</f>
-        <v>0.9375</v>
+      <c r="A29" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="C29" s="46" t="n">
+        <v>1650</v>
+      </c>
+      <c r="D29" s="46" t="n">
+        <v>1650</v>
+      </c>
+      <c r="E29" s="46" t="n">
+        <v>1623</v>
+      </c>
+      <c r="F29" s="46" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <f aca="false">F29/C29</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="C30" s="46" t="n">
+        <v>1950000</v>
+      </c>
+      <c r="D30" s="46" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="E30" s="46" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="F30" s="46" t="n">
+        <v>900700</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <f aca="false">F30/C30</f>
+        <v>0.461897435897436</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="26" t="s">
-        <v>270</v>
+      <c r="A31" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="C31" s="46" t="n">
+        <v>225000</v>
+      </c>
+      <c r="D31" s="46" t="n">
+        <v>185000</v>
+      </c>
+      <c r="E31" s="46" t="n">
+        <v>210000</v>
+      </c>
+      <c r="F31" s="46" t="n">
+        <v>114632</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <f aca="false">F31/C31</f>
+        <v>0.509475555555556</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="C32" s="46" t="n">
+        <v>660000</v>
+      </c>
+      <c r="D32" s="46" t="n">
+        <v>580000</v>
+      </c>
+      <c r="E32" s="46" t="n">
+        <v>570000</v>
+      </c>
+      <c r="F32" s="46" t="n">
+        <v>472000</v>
+      </c>
+      <c r="G32" s="14" t="n">
+        <f aca="false">F32/C32</f>
+        <v>0.715151515151515</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>320</v>
+      </c>
+      <c r="C33" s="46" t="n">
+        <v>114</v>
+      </c>
+      <c r="D33" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <f aca="false">F33/C33</f>
+        <v>0.0263157894736842</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="26" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="26" t="s">
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -6276,6 +7096,251 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="B2:C31"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="1" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="52" t="s">
+        <v>323</v>
+      </c>
+      <c r="C2" s="53" t="n">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="52" t="s">
+        <v>324</v>
+      </c>
+      <c r="C3" s="54" t="n">
+        <v>2.7283</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="52" t="s">
+        <v>325</v>
+      </c>
+      <c r="C4" s="55" t="n">
+        <f aca="false">C2*C3</f>
+        <v>2149.9004</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="52" t="s">
+        <v>326</v>
+      </c>
+      <c r="C5" s="48" t="n">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="52" t="s">
+        <v>327</v>
+      </c>
+      <c r="C6" s="56" t="n">
+        <v>273.5</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="52" t="s">
+        <v>328</v>
+      </c>
+      <c r="C7" s="57" t="n">
+        <f aca="false">'P&amp;L'!H180</f>
+        <v>49.715</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="52" t="s">
+        <v>329</v>
+      </c>
+      <c r="C8" s="48" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="52" t="s">
+        <v>330</v>
+      </c>
+      <c r="C9" s="58" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="52" t="s">
+        <v>331</v>
+      </c>
+      <c r="C10" s="49" t="n">
+        <f aca="false">C8-C9-C7</f>
+        <v>218.285</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="52" t="s">
+        <v>332</v>
+      </c>
+      <c r="C11" s="55" t="n">
+        <f aca="false">C4-C10</f>
+        <v>1931.6154</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="4" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="52" t="s">
+        <v>334</v>
+      </c>
+      <c r="C14" s="50" t="n">
+        <f aca="false">C11/'P&amp;L'!H3</f>
+        <v>39.079376062151</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="52" t="s">
+        <v>335</v>
+      </c>
+      <c r="C15" s="50" t="n">
+        <f aca="false">C2/129.23</f>
+        <v>6.09765534318657</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="52" t="s">
+        <v>336</v>
+      </c>
+      <c r="C16" s="59" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="4" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="52" t="s">
+        <v>339</v>
+      </c>
+      <c r="C19" s="58" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="52" t="s">
+        <v>340</v>
+      </c>
+      <c r="C20" s="58" t="n">
+        <v>1.64</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="52" t="s">
+        <v>341</v>
+      </c>
+      <c r="C21" s="55" t="n">
+        <f aca="false">C19*12*C20</f>
+        <v>787.2</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="C22" s="60" t="n">
+        <f aca="false">SUM(Segments!C4:C6)</f>
+        <v>44.72</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="52" t="s">
+        <v>343</v>
+      </c>
+      <c r="C23" s="55" t="n">
+        <f aca="false">C21+C22</f>
+        <v>831.92</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="52" t="s">
+        <v>344</v>
+      </c>
+      <c r="C24" s="61" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="52" t="s">
+        <v>345</v>
+      </c>
+      <c r="C25" s="55" t="n">
+        <f aca="false">C23*C24</f>
+        <v>83.192</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="52" t="s">
+        <v>346</v>
+      </c>
+      <c r="C26" s="50" t="n">
+        <f aca="false">C4/C25</f>
+        <v>25.8426339071065</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="52" t="s">
+        <v>347</v>
+      </c>
+      <c r="C27" s="55" t="n">
+        <f aca="false">C19*12</f>
+        <v>480</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="52" t="s">
+        <v>348</v>
+      </c>
+      <c r="C28" s="62" t="n">
+        <f aca="false">Segments!C20/C27*12</f>
+        <v>14.1</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="52" t="s">
+        <v>349</v>
+      </c>
+      <c r="C29" s="63" t="n">
+        <f aca="false">450/C27</f>
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="26" t="s">
+        <v>350</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -6285,74 +7350,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="B1" s="50" t="s">
-        <v>272</v>
+        <v>351</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>352</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="B2" s="50" t="s">
-        <v>274</v>
+        <v>353</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="B3" s="50" t="s">
-        <v>276</v>
+        <v>355</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="B4" s="50" t="s">
-        <v>278</v>
+        <v>357</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="B5" s="50" t="s">
-        <v>280</v>
+        <v>359</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="B6" s="50" t="s">
-        <v>282</v>
+        <v>361</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="B7" s="50" t="s">
-        <v>284</v>
+        <v>363</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="B8" s="50" t="s">
-        <v>286</v>
+        <v>365</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="B9" s="50" t="s">
-        <v>288</v>
+        <v>367</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>